<commit_message>
sheet export: page layout from rows_per_page; distinct fixture names
</commit_message>
<xml_diff>
--- a/fixtures/employees_punch_demo.xlsx
+++ b/fixtures/employees_punch_demo.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Zi Fong (device user 1)</t>
+          <t>Yeoh Kim Seng</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Wei Sheng binti Rahman</t>
+          <t>Wei Sheng Tan</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Nurul binti Rahman</t>
+          <t>Nurul Tan</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Chee Keong binti Rahman</t>
+          <t>Chee Keong Tan</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Mei Ling a/l Subramaniam</t>
+          <t>Mei Ling Tan</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Aung a/l Subramaniam</t>
+          <t>Aung Tan</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Chandran a/l Subramaniam</t>
+          <t>Chandran Tan</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Zubaidah Lim</t>
+          <t>Zubaidah Tan</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Kai Xin Lim</t>
+          <t>Kai Xin Tan</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hafiz Lim</t>
+          <t>Hafiz Tan</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Su Lin Wong</t>
+          <t>Su Lin Tan</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Arun Wong</t>
+          <t>Arun Tan</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Boon Hui Wong</t>
+          <t>Boon Hui Tan</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Farah Ko Min</t>
+          <t>Farah Tan</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Jia Hui Ko Min</t>
+          <t>Jia Hui Tan</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kumar Ko Min</t>
+          <t>Kumar Tan</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Lina a/l Muthu</t>
+          <t>Lina Tan</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Tze Yang a/l Muthu</t>
+          <t>Tze Yang Tan</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Ah Meng a/l Muthu</t>
+          <t>Poh Choo Tan</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Siti binti Osman</t>
+          <t>Zainal Tan</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Ravi binti Osman</t>
+          <t>Vimala Tan</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Wei Sheng binti Osman</t>
+          <t>Beng Huat Tan</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Nurul Chong</t>
+          <t>Rosnah Tan</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Chee Keong Chong</t>
+          <t>Sanjay Tan</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Mei Ling Chong</t>
+          <t>Yoke Lan Tan</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Aung Ismail</t>
+          <t>Idris Tan</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Chandran Ismail</t>
+          <t>Kalai Tan</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Zubaidah Ismail</t>
+          <t>Cheng Hoe Tan</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Kai Xin Tan</t>
+          <t>Norhayati Tan</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Hafiz Tan</t>
+          <t>Prakash Tan</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Su Lin Tan</t>
+          <t>Swee Lian Tan</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Arun binti Rahman</t>
+          <t>Faizal Tan</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Boon Hui binti Rahman</t>
+          <t>Devi Tan</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Farah binti Rahman</t>
+          <t>Kok Wai Tan</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Jia Hui a/l Subramaniam</t>
+          <t>Anisah Tan</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Kumar a/l Subramaniam</t>
+          <t>Ganesan Tan</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Lina a/l Subramaniam</t>
+          <t>Peik Ying Tan</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Tze Yang Lim</t>
+          <t>Rahim Tan</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Ah Meng Lim</t>
+          <t>Ah Meng binti Rahman</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Siti Lim</t>
+          <t>Siti binti Rahman</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Ravi Wong</t>
+          <t>Ravi binti Rahman</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Wei Sheng Wong</t>
+          <t>Wei Sheng binti Rahman</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Nurul Wong</t>
+          <t>Nurul binti Rahman</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Chee Keong Ko Min</t>
+          <t>Chee Keong binti Rahman</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Mei Ling Ko Min</t>
+          <t>Mei Ling binti Rahman</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Aung Ko Min</t>
+          <t>Aung binti Rahman</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Chandran a/l Muthu</t>
+          <t>Chandran binti Rahman</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Zubaidah a/l Muthu</t>
+          <t>Zubaidah binti Rahman</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Kai Xin a/l Muthu</t>
+          <t>Kai Xin binti Rahman</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Ah Meng Tan</t>
+          <t>Poh Choo binti Rahman</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Siti Tan</t>
+          <t>Zainal binti Rahman</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Ravi Tan</t>
+          <t>Vimala binti Rahman</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2828,7 +2828,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Wei Sheng binti Rahman</t>
+          <t>Beng Huat binti Rahman</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">

</xml_diff>